<commit_message>
Add Aasted US change point figures and organized outputs
</commit_message>
<xml_diff>
--- a/outputs/aasted3_run_comparison/summary/aasted3_reference_based_comparison_summary.xlsx
+++ b/outputs/aasted3_run_comparison/summary/aasted3_reference_based_comparison_summary.xlsx
@@ -12846,7 +12846,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y32"/>
+  <dimension ref="A1:AF32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12856,24 +12856,31 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="23" customWidth="1" min="8" max="8"/>
-    <col width="21" customWidth="1" min="9" max="9"/>
-    <col width="26" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
-    <col width="29" customWidth="1" min="12" max="12"/>
-    <col width="34" customWidth="1" min="13" max="13"/>
-    <col width="30" customWidth="1" min="14" max="14"/>
-    <col width="34" customWidth="1" min="15" max="15"/>
-    <col width="34" customWidth="1" min="16" max="16"/>
-    <col width="34" customWidth="1" min="17" max="17"/>
-    <col width="20" customWidth="1" min="18" max="18"/>
-    <col width="23" customWidth="1" min="19" max="19"/>
-    <col width="22" customWidth="1" min="20" max="20"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="23" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="25" customWidth="1" min="13" max="13"/>
+    <col width="21" customWidth="1" min="14" max="14"/>
+    <col width="26" customWidth="1" min="15" max="15"/>
+    <col width="24" customWidth="1" min="16" max="16"/>
+    <col width="32" customWidth="1" min="17" max="17"/>
+    <col width="30" customWidth="1" min="18" max="18"/>
+    <col width="29" customWidth="1" min="19" max="19"/>
+    <col width="34" customWidth="1" min="20" max="20"/>
     <col width="30" customWidth="1" min="21" max="21"/>
     <col width="34" customWidth="1" min="22" max="22"/>
-    <col width="21" customWidth="1" min="23" max="23"/>
-    <col width="14" customWidth="1" min="24" max="24"/>
-    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="34" customWidth="1" min="23" max="23"/>
+    <col width="34" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="25" max="25"/>
+    <col width="23" customWidth="1" min="26" max="26"/>
+    <col width="22" customWidth="1" min="27" max="27"/>
+    <col width="30" customWidth="1" min="28" max="28"/>
+    <col width="34" customWidth="1" min="29" max="29"/>
+    <col width="21" customWidth="1" min="30" max="30"/>
+    <col width="14" customWidth="1" min="31" max="31"/>
+    <col width="14" customWidth="1" min="32" max="32"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -13578,90 +13585,125 @@
       </c>
       <c r="H28" s="1" t="inlineStr">
         <is>
+          <t>analysis_domain</t>
+        </is>
+      </c>
+      <c r="I28" s="1" t="inlineStr">
+        <is>
+          <t>analysis_window_start_s</t>
+        </is>
+      </c>
+      <c r="J28" s="1" t="inlineStr">
+        <is>
           <t>analysis_window_end_s</t>
         </is>
       </c>
-      <c r="I28" s="1" t="inlineStr">
+      <c r="K28" s="1" t="inlineStr">
+        <is>
+          <t>first_change_point_s</t>
+        </is>
+      </c>
+      <c r="L28" s="1" t="inlineStr">
+        <is>
+          <t>first_change_point_after_onset_s</t>
+        </is>
+      </c>
+      <c r="M28" s="1" t="inlineStr">
+        <is>
+          <t>first_change_point_zone</t>
+        </is>
+      </c>
+      <c r="N28" s="1" t="inlineStr">
         <is>
           <t>detachment_offset_s</t>
         </is>
       </c>
-      <c r="J28" s="1" t="inlineStr">
+      <c r="O28" s="1" t="inlineStr">
         <is>
           <t>detachment_offset_status</t>
         </is>
       </c>
-      <c r="K28" s="1" t="inlineStr">
+      <c r="P28" s="1" t="inlineStr">
         <is>
           <t>detachment_offset_zone</t>
         </is>
       </c>
-      <c r="L28" s="1" t="inlineStr">
+      <c r="Q28" s="1" t="inlineStr">
+        <is>
+          <t>detachment_offset_zone_start_s</t>
+        </is>
+      </c>
+      <c r="R28" s="1" t="inlineStr">
+        <is>
+          <t>detachment_offset_zone_end_s</t>
+        </is>
+      </c>
+      <c r="S28" s="1" t="inlineStr">
         <is>
           <t>demoulding_twisting_start_s</t>
         </is>
       </c>
-      <c r="M28" s="1" t="inlineStr">
+      <c r="T28" s="1" t="inlineStr">
         <is>
           <t>complete_detachment_before_demoulding</t>
         </is>
       </c>
-      <c r="N28" s="1" t="inlineStr">
+      <c r="U28" s="1" t="inlineStr">
         <is>
           <t>detachment_onset_to_offset_s</t>
         </is>
       </c>
-      <c r="O28" s="1" t="inlineStr">
+      <c r="V28" s="1" t="inlineStr">
         <is>
           <t>detachment_offset_minus_deposition_s</t>
         </is>
       </c>
-      <c r="P28" s="1" t="inlineStr">
+      <c r="W28" s="1" t="inlineStr">
         <is>
           <t>detachment_onset_minus_deposition_s</t>
         </is>
       </c>
-      <c r="Q28" s="1" t="inlineStr">
+      <c r="X28" s="1" t="inlineStr">
         <is>
           <t>crystallization_onset_minus_deposition_s</t>
         </is>
       </c>
-      <c r="R28" s="1" t="inlineStr">
+      <c r="Y28" s="1" t="inlineStr">
         <is>
           <t>reference_us_level</t>
         </is>
       </c>
-      <c r="S28" s="1" t="inlineStr">
+      <c r="Z28" s="1" t="inlineStr">
         <is>
           <t>threshold_10pct_lower</t>
         </is>
       </c>
-      <c r="T28" s="1" t="inlineStr">
+      <c r="AA28" s="1" t="inlineStr">
         <is>
           <t>us_level_at_decision</t>
         </is>
       </c>
-      <c r="U28" s="1" t="inlineStr">
+      <c r="AB28" s="1" t="inlineStr">
         <is>
           <t>change_points_detected_total</t>
         </is>
       </c>
-      <c r="V28" s="1" t="inlineStr">
+      <c r="AC28" s="1" t="inlineStr">
         <is>
           <t>change_points_until_detachment_or_last</t>
         </is>
       </c>
-      <c r="W28" s="1" t="inlineStr">
+      <c r="AD28" s="1" t="inlineStr">
         <is>
           <t>pattern_description</t>
         </is>
       </c>
-      <c r="X28" s="1" t="inlineStr">
+      <c r="AE28" s="1" t="inlineStr">
         <is>
           <t>method</t>
         </is>
       </c>
-      <c r="Y28" s="1" t="inlineStr">
+      <c r="AF28" s="1" t="inlineStr">
         <is>
           <t>source_file</t>
         </is>
@@ -13697,66 +13739,91 @@
       <c r="G29" t="n">
         <v>1454</v>
       </c>
-      <c r="H29" t="n">
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>detachment_onset_to_run_end</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>1454</v>
+      </c>
+      <c r="J29" t="n">
         <v>2213.480570077896</v>
       </c>
-      <c r="I29" t="n">
+      <c r="K29" t="n">
+        <v>1533.480596780777</v>
+      </c>
+      <c r="L29" t="n">
+        <v>79.48059678077652</v>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>less_periodic_cooling_2</t>
+        </is>
+      </c>
+      <c r="N29" t="n">
         <v>2073.480711936951</v>
       </c>
-      <c r="J29" t="inlineStr">
+      <c r="O29" t="inlineStr">
         <is>
           <t>complete_detachment_for_channel</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr">
+      <c r="P29" t="inlineStr">
         <is>
           <t>transition_2</t>
         </is>
       </c>
-      <c r="L29" t="n">
+      <c r="Q29" t="n">
+        <v>1976</v>
+      </c>
+      <c r="R29" t="n">
         <v>2118</v>
       </c>
-      <c r="M29" t="n">
+      <c r="S29" t="n">
+        <v>2118</v>
+      </c>
+      <c r="T29" t="n">
         <v>1</v>
       </c>
-      <c r="N29" t="n">
+      <c r="U29" t="n">
         <v>619.4807119369507</v>
       </c>
-      <c r="O29" t="n">
+      <c r="V29" t="n">
         <v>1789.480711936951</v>
       </c>
-      <c r="P29" t="n">
+      <c r="W29" t="n">
         <v>1170</v>
       </c>
-      <c r="Q29" t="n">
+      <c r="X29" t="n">
         <v>344</v>
       </c>
-      <c r="R29" t="n">
+      <c r="Y29" t="n">
         <v>0.9854422053609572</v>
       </c>
-      <c r="S29" t="n">
+      <c r="Z29" t="n">
         <v>0.8868979848248615</v>
       </c>
-      <c r="T29" t="n">
+      <c r="AA29" t="n">
         <v>0.9387736268774387</v>
       </c>
-      <c r="U29" t="n">
+      <c r="AB29" t="n">
         <v>2</v>
       </c>
-      <c r="V29" t="n">
+      <c r="AC29" t="n">
         <v>2</v>
       </c>
-      <c r="W29" t="inlineStr">
+      <c r="AD29" t="inlineStr">
         <is>
           <t>2 positive upward change point(s) from detachment onset to run end. First complete offset at 2073.5s.</t>
         </is>
       </c>
-      <c r="X29" t="inlineStr">
+      <c r="AE29" t="inlineStr">
         <is>
           <t>positive/upward local mean-shift change points on T7-corrected ultrasound; complete detachment if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
-      <c r="Y29" t="inlineStr">
+      <c r="AF29" t="inlineStr">
         <is>
           <t>aa3_trials_experimental_summary.xlsx</t>
         </is>
@@ -13792,66 +13859,91 @@
       <c r="G30" t="n">
         <v>1456</v>
       </c>
-      <c r="H30" t="n">
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>detachment_onset_to_run_end</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>1456</v>
+      </c>
+      <c r="J30" t="n">
         <v>2213.480570077896</v>
       </c>
-      <c r="I30" t="n">
+      <c r="K30" t="n">
+        <v>1517.48148560524</v>
+      </c>
+      <c r="L30" t="n">
+        <v>61.48148560523987</v>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>less_periodic_cooling_2</t>
+        </is>
+      </c>
+      <c r="N30" t="n">
         <v>2071.500448465347</v>
       </c>
-      <c r="J30" t="inlineStr">
+      <c r="O30" t="inlineStr">
         <is>
           <t>complete_detachment_for_channel</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr">
+      <c r="P30" t="inlineStr">
         <is>
           <t>transition_2</t>
         </is>
       </c>
-      <c r="L30" t="n">
+      <c r="Q30" t="n">
+        <v>1976</v>
+      </c>
+      <c r="R30" t="n">
         <v>2118</v>
       </c>
-      <c r="M30" t="n">
+      <c r="S30" t="n">
+        <v>2118</v>
+      </c>
+      <c r="T30" t="n">
         <v>1</v>
       </c>
-      <c r="N30" t="n">
+      <c r="U30" t="n">
         <v>615.5004484653473</v>
       </c>
-      <c r="O30" t="n">
+      <c r="V30" t="n">
         <v>1787.500448465347</v>
       </c>
-      <c r="P30" t="n">
+      <c r="W30" t="n">
         <v>1172</v>
       </c>
-      <c r="Q30" t="n">
+      <c r="X30" t="n">
         <v>342</v>
       </c>
-      <c r="R30" t="n">
+      <c r="Y30" t="n">
         <v>0.8087176470762016</v>
       </c>
-      <c r="S30" t="n">
+      <c r="Z30" t="n">
         <v>0.7278458823685815</v>
       </c>
-      <c r="T30" t="n">
+      <c r="AA30" t="n">
         <v>0.82536306643459</v>
       </c>
-      <c r="U30" t="n">
+      <c r="AB30" t="n">
         <v>3</v>
       </c>
-      <c r="V30" t="n">
+      <c r="AC30" t="n">
         <v>3</v>
       </c>
-      <c r="W30" t="inlineStr">
+      <c r="AD30" t="inlineStr">
         <is>
           <t>3 positive upward change point(s) from detachment onset to run end. First complete offset at 2071.5s.</t>
         </is>
       </c>
-      <c r="X30" t="inlineStr">
+      <c r="AE30" t="inlineStr">
         <is>
           <t>positive/upward local mean-shift change points on T7-corrected ultrasound; complete detachment if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
-      <c r="Y30" t="inlineStr">
+      <c r="AF30" t="inlineStr">
         <is>
           <t>aa3_trials_experimental_summary.xlsx</t>
         </is>
@@ -13887,66 +13979,91 @@
       <c r="G31" t="n">
         <v>1430</v>
       </c>
-      <c r="H31" t="n">
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>detachment_onset_to_run_end</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>1430</v>
+      </c>
+      <c r="J31" t="n">
         <v>1868.234316587448</v>
       </c>
-      <c r="I31" t="n">
+      <c r="K31" t="n">
+        <v>1523.292253017426</v>
+      </c>
+      <c r="L31" t="n">
+        <v>93.29225301742554</v>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>less_periodic_cooling_2</t>
+        </is>
+      </c>
+      <c r="N31" t="n">
         <v>1755.292186975479</v>
       </c>
-      <c r="J31" t="inlineStr">
+      <c r="O31" t="inlineStr">
         <is>
           <t>complete_detachment_for_channel</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr">
+      <c r="P31" t="inlineStr">
         <is>
           <t>transition_2</t>
         </is>
       </c>
-      <c r="L31" t="n">
+      <c r="Q31" t="n">
+        <v>1629</v>
+      </c>
+      <c r="R31" t="n">
         <v>1792</v>
       </c>
-      <c r="M31" t="n">
+      <c r="S31" t="n">
+        <v>1792</v>
+      </c>
+      <c r="T31" t="n">
         <v>1</v>
       </c>
-      <c r="N31" t="n">
+      <c r="U31" t="n">
         <v>325.2921869754791</v>
       </c>
-      <c r="O31" t="n">
+      <c r="V31" t="n">
         <v>1469.292186975479</v>
       </c>
-      <c r="P31" t="n">
+      <c r="W31" t="n">
         <v>1144</v>
       </c>
-      <c r="Q31" t="n">
+      <c r="X31" t="n">
         <v>344</v>
       </c>
-      <c r="R31" t="n">
+      <c r="Y31" t="n">
         <v>0.9886593692731603</v>
       </c>
-      <c r="S31" t="n">
+      <c r="Z31" t="n">
         <v>0.8897934323458443</v>
       </c>
-      <c r="T31" t="n">
+      <c r="AA31" t="n">
         <v>0.9108031549980742</v>
       </c>
-      <c r="U31" t="n">
+      <c r="AB31" t="n">
         <v>2</v>
       </c>
-      <c r="V31" t="n">
+      <c r="AC31" t="n">
         <v>2</v>
       </c>
-      <c r="W31" t="inlineStr">
+      <c r="AD31" t="inlineStr">
         <is>
           <t>2 positive upward change point(s) from detachment onset to run end. First complete offset at 1755.3s.</t>
         </is>
       </c>
-      <c r="X31" t="inlineStr">
+      <c r="AE31" t="inlineStr">
         <is>
           <t>positive/upward local mean-shift change points on T7-corrected ultrasound; complete detachment if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
-      <c r="Y31" t="inlineStr">
+      <c r="AF31" t="inlineStr">
         <is>
           <t>aa3_trials_experimental_summary.xlsx</t>
         </is>
@@ -13982,66 +14099,91 @@
       <c r="G32" t="n">
         <v>1430</v>
       </c>
-      <c r="H32" t="n">
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>detachment_onset_to_run_end</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>1430</v>
+      </c>
+      <c r="J32" t="n">
         <v>1868.234316587448</v>
       </c>
-      <c r="I32" t="n">
+      <c r="K32" t="n">
+        <v>1643.292067527771</v>
+      </c>
+      <c r="L32" t="n">
+        <v>213.292067527771</v>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>transition_2</t>
+        </is>
+      </c>
+      <c r="N32" t="n">
         <v>1757.292216777802</v>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="O32" t="inlineStr">
         <is>
           <t>complete_detachment_for_channel</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr">
+      <c r="P32" t="inlineStr">
         <is>
           <t>transition_2</t>
         </is>
       </c>
-      <c r="L32" t="n">
+      <c r="Q32" t="n">
+        <v>1629</v>
+      </c>
+      <c r="R32" t="n">
         <v>1792</v>
       </c>
-      <c r="M32" t="n">
+      <c r="S32" t="n">
+        <v>1792</v>
+      </c>
+      <c r="T32" t="n">
         <v>1</v>
       </c>
-      <c r="N32" t="n">
+      <c r="U32" t="n">
         <v>327.2922167778015</v>
       </c>
-      <c r="O32" t="n">
+      <c r="V32" t="n">
         <v>1471.292216777802</v>
       </c>
-      <c r="P32" t="n">
+      <c r="W32" t="n">
         <v>1144</v>
       </c>
-      <c r="Q32" t="n">
+      <c r="X32" t="n">
         <v>344</v>
       </c>
-      <c r="R32" t="n">
+      <c r="Y32" t="n">
         <v>0.8195161085032753</v>
       </c>
-      <c r="S32" t="n">
+      <c r="Z32" t="n">
         <v>0.7375644976529477</v>
       </c>
-      <c r="T32" t="n">
+      <c r="AA32" t="n">
         <v>0.8063564620894778</v>
       </c>
-      <c r="U32" t="n">
+      <c r="AB32" t="n">
         <v>2</v>
       </c>
-      <c r="V32" t="n">
+      <c r="AC32" t="n">
         <v>2</v>
       </c>
-      <c r="W32" t="inlineStr">
+      <c r="AD32" t="inlineStr">
         <is>
           <t>2 positive upward change point(s) from detachment onset to run end. First complete offset at 1757.3s.</t>
         </is>
       </c>
-      <c r="X32" t="inlineStr">
+      <c r="AE32" t="inlineStr">
         <is>
           <t>positive/upward local mean-shift change points on T7-corrected ultrasound; complete detachment if US at change point &gt;= 10%-below-pre-deposition-reference threshold</t>
         </is>
       </c>
-      <c r="Y32" t="inlineStr">
+      <c r="AF32" t="inlineStr">
         <is>
           <t>aa3_trials_experimental_summary.xlsx</t>
         </is>

</xml_diff>